<commit_message>
Reframe PCL MDE: remove target lift, MDE is the output
No target lift or OK/NOT OK — MDE shows the minimum detectable
difference between placements. Business decides if that's small enough.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcl_mde_calculator.xlsx
+++ b/pcl_mde_calculator.xlsx
@@ -16,12 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.0000%"/>
-    <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +34,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00404040"/>
     </font>
   </fonts>
   <fills count="6">
@@ -87,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -108,35 +111,16 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="00006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="00C6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="00FF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="00FFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -498,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L44"/>
+  <dimension ref="A2:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -510,9 +494,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -530,8 +512,6 @@
       <c r="H2" s="1" t="n"/>
       <c r="I2" s="1" t="n"/>
       <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
-      <c r="L2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="3" t="inlineStr">
@@ -636,16 +616,6 @@
       </c>
       <c r="C9" s="5" t="n">
         <v>0.8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Target Lift</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>0.05</v>
       </c>
     </row>
     <row r="11">
@@ -663,8 +633,6 @@
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
       <c r="J11" s="1" t="n"/>
-      <c r="K11" s="1" t="n"/>
-      <c r="L11" s="1" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
@@ -703,8 +671,6 @@
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="n"/>
-      <c r="K16" s="1" t="n"/>
-      <c r="L16" s="1" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr"/>
@@ -839,8 +805,6 @@
       <c r="H23" s="1" t="n"/>
       <c r="I23" s="1" t="n"/>
       <c r="J23" s="1" t="n"/>
-      <c r="K23" s="1" t="n"/>
-      <c r="L23" s="1" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
@@ -890,17 +854,7 @@
       </c>
       <c r="J24" s="15" t="inlineStr">
         <is>
-          <t>Target Lift</t>
-        </is>
-      </c>
-      <c r="K24" s="15" t="inlineStr">
-        <is>
-          <t>Headroom</t>
-        </is>
-      </c>
-      <c r="L24" s="15" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Interpretation</t>
         </is>
       </c>
     </row>
@@ -942,16 +896,8 @@
         <f>ROUND(($C$13+$C$14)*SQRT(H25*(1-H25)*(1/D25+1/E25)),4)</f>
         <v/>
       </c>
-      <c r="J25" s="12">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="K25" s="18">
-        <f>J25/I25</f>
-        <v/>
-      </c>
-      <c r="L25" s="13">
-        <f>IF(I25&lt;J25,"OK","NOT OK")</f>
+      <c r="J25" s="18">
+        <f>"Can detect differences "&amp;CHAR(8805)&amp;" "&amp;TEXT(I25*100,"0.00")&amp;" pp"</f>
         <v/>
       </c>
     </row>
@@ -993,16 +939,8 @@
         <f>ROUND(($C$13+$C$14)*SQRT(H26*(1-H26)*(1/D26+1/E26)),4)</f>
         <v/>
       </c>
-      <c r="J26" s="12">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="K26" s="18">
-        <f>J26/I26</f>
-        <v/>
-      </c>
-      <c r="L26" s="13">
-        <f>IF(I26&lt;J26,"OK","NOT OK")</f>
+      <c r="J26" s="18">
+        <f>"Can detect differences "&amp;CHAR(8805)&amp;" "&amp;TEXT(I26*100,"0.00")&amp;" pp"</f>
         <v/>
       </c>
     </row>
@@ -1044,16 +982,8 @@
         <f>ROUND(($C$13+$C$14)*SQRT(H27*(1-H27)*(1/D27+1/E27)),4)</f>
         <v/>
       </c>
-      <c r="J27" s="12">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="K27" s="18">
-        <f>J27/I27</f>
-        <v/>
-      </c>
-      <c r="L27" s="13">
-        <f>IF(I27&lt;J27,"OK","NOT OK")</f>
+      <c r="J27" s="18">
+        <f>"Can detect differences "&amp;CHAR(8805)&amp;" "&amp;TEXT(I27*100,"0.00")&amp;" pp"</f>
         <v/>
       </c>
     </row>
@@ -1095,140 +1025,80 @@
         <f>ROUND(($C$13+$C$14)*SQRT(H28*(1-H28)*(1/D28+1/E28)),4)</f>
         <v/>
       </c>
-      <c r="J28" s="12">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="K28" s="18">
-        <f>J28/I28</f>
-        <v/>
-      </c>
-      <c r="L28" s="13">
-        <f>IF(I28&lt;J28,"OK","NOT OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="n"/>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="J28" s="18">
+        <f>"Can detect differences "&amp;CHAR(8805)&amp;" "&amp;TEXT(I28*100,"0.00")&amp;" pp"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>The MDE is the minimum lift (in percentage points) detectable with 80% power at 5% significance. If the actual difference between placements is smaller than the MDE, this test will not reliably detect it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n"/>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Stress Test Scenarios</t>
         </is>
       </c>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
-      <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="1" t="n"/>
-      <c r="H31" s="1" t="n"/>
-      <c r="I31" s="1" t="n"/>
-      <c r="J31" s="1" t="n"/>
-      <c r="K31" s="1" t="n"/>
-      <c r="L31" s="1" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="15" t="inlineStr"/>
-      <c r="B32" s="15" t="inlineStr">
+      <c r="C32" s="1" t="n"/>
+      <c r="D32" s="1" t="n"/>
+      <c r="E32" s="1" t="n"/>
+      <c r="F32" s="1" t="n"/>
+      <c r="G32" s="1" t="n"/>
+      <c r="H32" s="1" t="n"/>
+      <c r="I32" s="1" t="n"/>
+      <c r="J32" s="1" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr"/>
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>Baseline RR</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>Comp 1 MDE</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>Comp 2 MDE</t>
         </is>
       </c>
-      <c r="F32" s="15" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>Comp 3 MDE</t>
         </is>
       </c>
-      <c r="G32" s="15" t="inlineStr">
+      <c r="G33" s="15" t="inlineStr">
         <is>
           <t>Comp 4 MDE</t>
         </is>
       </c>
-      <c r="H32" s="15" t="inlineStr">
+      <c r="H33" s="15" t="inlineStr">
         <is>
           <t>Worst Case MDE</t>
         </is>
-      </c>
-      <c r="I32" s="15" t="inlineStr">
-        <is>
-          <t>Target Lift</t>
-        </is>
-      </c>
-      <c r="J32" s="15" t="inlineStr">
-        <is>
-          <t>Headroom</t>
-        </is>
-      </c>
-      <c r="K32" s="15" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Pessimistic</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="D33" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C33*(1-C33)*(1/C19+1/C20)),4)</f>
-        <v/>
-      </c>
-      <c r="E33" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C33*(1-C33)*(1/C19+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="F33" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C33*(1-C33)*(1/C20+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="G33" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C33*(1-C33)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
-        <v/>
-      </c>
-      <c r="H33" s="17">
-        <f>MAX(D33:G33)</f>
-        <v/>
-      </c>
-      <c r="I33" s="12">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="J33" s="18">
-        <f>I33/H33</f>
-        <v/>
-      </c>
-      <c r="K33" s="13">
-        <f>IF(H33&lt;I33,"OK","NOT OK")</f>
-        <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Pessimistic</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="D34" s="17">
         <f>ROUND(($C$13+$C$14)*SQRT(C34*(1-C34)*(1/C19+1/C20)),4)</f>
@@ -1250,27 +1120,15 @@
         <f>MAX(D34:G34)</f>
         <v/>
       </c>
-      <c r="I34" s="12">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="J34" s="18">
-        <f>I34/H34</f>
-        <v/>
-      </c>
-      <c r="K34" s="13">
-        <f>IF(H34&lt;I34,"OK","NOT OK")</f>
-        <v/>
-      </c>
     </row>
     <row r="35">
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Optimistic</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="D35" s="17">
         <f>ROUND(($C$13+$C$14)*SQRT(C35*(1-C35)*(1/C19+1/C20)),4)</f>
@@ -1292,103 +1150,106 @@
         <f>MAX(D35:G35)</f>
         <v/>
       </c>
-      <c r="I35" s="12">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="J35" s="18">
-        <f>I35/H35</f>
-        <v/>
-      </c>
-      <c r="K35" s="13">
-        <f>IF(H35&lt;I35,"OK","NOT OK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n"/>
-      <c r="B37" s="2" t="inlineStr">
+    </row>
+    <row r="36">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Optimistic</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D36" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/C19+1/C20)),4)</f>
+        <v/>
+      </c>
+      <c r="E36" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/C19+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="F36" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/C20+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="G36" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
+        <v/>
+      </c>
+      <c r="H36" s="17">
+        <f>MAX(D36:G36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C37" s="1" t="n"/>
-      <c r="D37" s="1" t="n"/>
-      <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="n"/>
-      <c r="G37" s="1" t="n"/>
-      <c r="H37" s="1" t="n"/>
-      <c r="I37" s="1" t="n"/>
-      <c r="J37" s="1" t="n"/>
-      <c r="K37" s="1" t="n"/>
-      <c r="L37" s="1" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>1. No control group — champion/challenger placement test.</t>
-        </is>
-      </c>
+      <c r="C38" s="1" t="n"/>
+      <c r="D38" s="1" t="n"/>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="1" t="n"/>
+      <c r="J38" s="1" t="n"/>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>2. Everyone gets the PCL offer — variable is WHERE they see it.</t>
+          <t>1. No control group — champion/challenger placement test.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>3. Baseline RR = all-channel population-level rate (not mobile share).</t>
+          <t>2. Everyone gets the PCL offer — variable is WHERE they see it.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>4. PCL mnemonic confirmed by Daniel Chin (was PLI).</t>
+          <t>3. Baseline RR = all-channel population-level rate (not mobile share).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>5. Green cells are editable — change them to see recalculations.</t>
+          <t>4. PCL mnemonic confirmed by Daniel Chin (was PLI).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>6. MDE formula: (Za + Zb) * SQRT(p0 * (1-p0) * (1/n1 + 1/n2)).</t>
+          <t>5. Green cells are editable — change them to see recalculations.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
+          <t>6. MDE formula: (Za + Zb) * SQRT(p0 * (1-p0) * (1/n1 + 1/n2)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
           <t>7. If reporting all 4 comparisons, consider Bonferroni correction (alpha/4 = 1.25%).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L25:L28">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"NOT OK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K33:K35">
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
-      <formula>"NOT OK"</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <mergeCells count="1">
+    <mergeCell ref="B30:J30"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update PCL MDE: 7 comparisons (pairwise + each-vs-rest + conservative)
Added 3 each-vs-rest comparisons, Bonferroni note, expanded stress test.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcl_mde_calculator.xlsx
+++ b/pcl_mde_calculator.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <i val="1"/>
@@ -90,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +120,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J45"/>
+  <dimension ref="A2:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -495,6 +503,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -907,7 +916,7 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>Sales Model vs Product Page</t>
+          <t>Sales Model vs Product Page Champion</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -950,7 +959,7 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>Mobile Dashboard vs Product Page</t>
+          <t>Mobile Dashboard vs Product Page Champion</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
@@ -993,20 +1002,20 @@
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>Smallest Arm vs Rest (conservative)</t>
+          <t>Sales Model vs (Dashboard + Product Page)</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Did winning placement outperform others?</t>
+          <t>Did Sales Model outperform the other two combined?</t>
         </is>
       </c>
       <c r="D28" s="14">
-        <f>MIN(C19:C21)</f>
+        <f>C19</f>
         <v/>
       </c>
       <c r="E28" s="14">
-        <f>C3-MIN(C19:C21)</f>
+        <f>C20+C21</f>
         <v/>
       </c>
       <c r="F28" s="14">
@@ -1030,225 +1039,417 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="40" customHeight="1">
-      <c r="B30" s="19" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Mobile Dashboard vs (Sales Model + Product Page)</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Did Dashboard outperform the other two combined?</t>
+        </is>
+      </c>
+      <c r="D29" s="14">
+        <f>C20</f>
+        <v/>
+      </c>
+      <c r="E29" s="14">
+        <f>C19+C21</f>
+        <v/>
+      </c>
+      <c r="F29" s="14">
+        <f>D29+E29</f>
+        <v/>
+      </c>
+      <c r="G29" s="16">
+        <f>D29/E29</f>
+        <v/>
+      </c>
+      <c r="H29" s="12">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="I29" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(H29*(1-H29)*(1/D29+1/E29)),4)</f>
+        <v/>
+      </c>
+      <c r="J29" s="18">
+        <f>"Can detect differences "&amp;CHAR(8805)&amp;" "&amp;TEXT(I29*100,"0.00")&amp;" pp"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Product Page vs (Sales Model + Dashboard)</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Did Product Page outperform the other two combined?</t>
+        </is>
+      </c>
+      <c r="D30" s="14">
+        <f>C21</f>
+        <v/>
+      </c>
+      <c r="E30" s="14">
+        <f>C19+C20</f>
+        <v/>
+      </c>
+      <c r="F30" s="14">
+        <f>D30+E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="16">
+        <f>D30/E30</f>
+        <v/>
+      </c>
+      <c r="H30" s="12">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="I30" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(H30*(1-H30)*(1/D30+1/E30)),4)</f>
+        <v/>
+      </c>
+      <c r="J30" s="18">
+        <f>"Can detect differences "&amp;CHAR(8805)&amp;" "&amp;TEXT(I30*100,"0.00")&amp;" pp"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Smallest Arm vs Rest (conservative)</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Conservative worst-case: can we detect differences for the smallest group?</t>
+        </is>
+      </c>
+      <c r="D31" s="14">
+        <f>MIN(C19:C21)</f>
+        <v/>
+      </c>
+      <c r="E31" s="14">
+        <f>C3-MIN(C19:C21)</f>
+        <v/>
+      </c>
+      <c r="F31" s="14">
+        <f>D31+E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="16">
+        <f>D31/E31</f>
+        <v/>
+      </c>
+      <c r="H31" s="12">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="I31" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(H31*(1-H31)*(1/D31+1/E31)),4)</f>
+        <v/>
+      </c>
+      <c r="J31" s="18">
+        <f>"Can detect differences "&amp;CHAR(8805)&amp;" "&amp;TEXT(I31*100,"0.00")&amp;" pp"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="35" customHeight="1">
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>With 7 comparisons, Bonferroni-adjusted significance = 5%/7 ≈ 0.71% per comparison (Za ≈ 2.4573). MDE increases slightly but remains small given sample sizes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>The MDE is the minimum lift (in percentage points) detectable with 80% power at 5% significance. If the actual difference between placements is smaller than the MDE, this test will not reliably detect it.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="n"/>
-      <c r="B32" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="1" t="n"/>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Stress Test Scenarios</t>
         </is>
       </c>
-      <c r="C32" s="1" t="n"/>
-      <c r="D32" s="1" t="n"/>
-      <c r="E32" s="1" t="n"/>
-      <c r="F32" s="1" t="n"/>
-      <c r="G32" s="1" t="n"/>
-      <c r="H32" s="1" t="n"/>
-      <c r="I32" s="1" t="n"/>
-      <c r="J32" s="1" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr"/>
-      <c r="B33" s="15" t="inlineStr">
+      <c r="C35" s="1" t="n"/>
+      <c r="D35" s="1" t="n"/>
+      <c r="E35" s="1" t="n"/>
+      <c r="F35" s="1" t="n"/>
+      <c r="G35" s="1" t="n"/>
+      <c r="H35" s="1" t="n"/>
+      <c r="I35" s="1" t="n"/>
+      <c r="J35" s="1" t="n"/>
+      <c r="K35" s="1" t="n"/>
+      <c r="L35" s="1" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr"/>
+      <c r="B36" s="15" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>Baseline RR</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>Comp 1 MDE</t>
         </is>
       </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E36" s="15" t="inlineStr">
         <is>
           <t>Comp 2 MDE</t>
         </is>
       </c>
-      <c r="F33" s="15" t="inlineStr">
+      <c r="F36" s="15" t="inlineStr">
         <is>
           <t>Comp 3 MDE</t>
         </is>
       </c>
-      <c r="G33" s="15" t="inlineStr">
+      <c r="G36" s="15" t="inlineStr">
         <is>
           <t>Comp 4 MDE</t>
         </is>
       </c>
-      <c r="H33" s="15" t="inlineStr">
+      <c r="H36" s="15" t="inlineStr">
+        <is>
+          <t>Comp 5 MDE</t>
+        </is>
+      </c>
+      <c r="I36" s="15" t="inlineStr">
+        <is>
+          <t>Comp 6 MDE</t>
+        </is>
+      </c>
+      <c r="J36" s="15" t="inlineStr">
+        <is>
+          <t>Comp 7 MDE</t>
+        </is>
+      </c>
+      <c r="K36" s="15" t="inlineStr">
         <is>
           <t>Worst Case MDE</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="13" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Pessimistic</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
+      <c r="C37" s="11" t="n">
         <v>0.14</v>
       </c>
-      <c r="D34" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C34*(1-C34)*(1/C19+1/C20)),4)</f>
-        <v/>
-      </c>
-      <c r="E34" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C34*(1-C34)*(1/C19+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="F34" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C34*(1-C34)*(1/C20+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="G34" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C34*(1-C34)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
-        <v/>
-      </c>
-      <c r="H34" s="17">
-        <f>MAX(D34:G34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="13" t="inlineStr">
+      <c r="D37" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C37*(1-C37)*(1/C19+1/C20)),4)</f>
+        <v/>
+      </c>
+      <c r="E37" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C37*(1-C37)*(1/C19+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="F37" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C37*(1-C37)*(1/C20+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="G37" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C37*(1-C37)*(1/C19+1/(C20+C21))),4)</f>
+        <v/>
+      </c>
+      <c r="H37" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C37*(1-C37)*(1/C20+1/(C19+C21))),4)</f>
+        <v/>
+      </c>
+      <c r="I37" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C37*(1-C37)*(1/C21+1/(C19+C20))),4)</f>
+        <v/>
+      </c>
+      <c r="J37" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C37*(1-C37)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
+        <v/>
+      </c>
+      <c r="K37" s="17">
+        <f>MAX(D37:J37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
+      <c r="C38" s="11" t="n">
         <v>0.15</v>
       </c>
-      <c r="D35" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C35*(1-C35)*(1/C19+1/C20)),4)</f>
-        <v/>
-      </c>
-      <c r="E35" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C35*(1-C35)*(1/C19+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="F35" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C35*(1-C35)*(1/C20+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="G35" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C35*(1-C35)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
-        <v/>
-      </c>
-      <c r="H35" s="17">
-        <f>MAX(D35:G35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="13" t="inlineStr">
+      <c r="D38" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C38*(1-C38)*(1/C19+1/C20)),4)</f>
+        <v/>
+      </c>
+      <c r="E38" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C38*(1-C38)*(1/C19+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="F38" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C38*(1-C38)*(1/C20+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="G38" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C38*(1-C38)*(1/C19+1/(C20+C21))),4)</f>
+        <v/>
+      </c>
+      <c r="H38" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C38*(1-C38)*(1/C20+1/(C19+C21))),4)</f>
+        <v/>
+      </c>
+      <c r="I38" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C38*(1-C38)*(1/C21+1/(C19+C20))),4)</f>
+        <v/>
+      </c>
+      <c r="J38" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C38*(1-C38)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
+        <v/>
+      </c>
+      <c r="K38" s="17">
+        <f>MAX(D38:J38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
+      <c r="C39" s="11" t="n">
         <v>0.22</v>
       </c>
-      <c r="D36" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/C19+1/C20)),4)</f>
-        <v/>
-      </c>
-      <c r="E36" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/C19+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="F36" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/C20+1/C21)),4)</f>
-        <v/>
-      </c>
-      <c r="G36" s="17">
-        <f>ROUND(($C$13+$C$14)*SQRT(C36*(1-C36)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
-        <v/>
-      </c>
-      <c r="H36" s="17">
-        <f>MAX(D36:G36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="D39" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C39*(1-C39)*(1/C19+1/C20)),4)</f>
+        <v/>
+      </c>
+      <c r="E39" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C39*(1-C39)*(1/C19+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="F39" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C39*(1-C39)*(1/C20+1/C21)),4)</f>
+        <v/>
+      </c>
+      <c r="G39" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C39*(1-C39)*(1/C19+1/(C20+C21))),4)</f>
+        <v/>
+      </c>
+      <c r="H39" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C39*(1-C39)*(1/C20+1/(C19+C21))),4)</f>
+        <v/>
+      </c>
+      <c r="I39" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C39*(1-C39)*(1/C21+1/(C19+C20))),4)</f>
+        <v/>
+      </c>
+      <c r="J39" s="17">
+        <f>ROUND(($C$13+$C$14)*SQRT(C39*(1-C39)*(1/(MIN(C19:C21))+1/(C3-MIN(C19:C21)))),4)</f>
+        <v/>
+      </c>
+      <c r="K39" s="17">
+        <f>MAX(D39:J39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C38" s="1" t="n"/>
-      <c r="D38" s="1" t="n"/>
-      <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="n"/>
-      <c r="G38" s="1" t="n"/>
-      <c r="H38" s="1" t="n"/>
-      <c r="I38" s="1" t="n"/>
-      <c r="J38" s="1" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>1. No control group — champion/challenger placement test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>2. Everyone gets the PCL offer — variable is WHERE they see it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>3. Baseline RR = all-channel population-level rate (not mobile share).</t>
-        </is>
-      </c>
+      <c r="C41" s="1" t="n"/>
+      <c r="D41" s="1" t="n"/>
+      <c r="E41" s="1" t="n"/>
+      <c r="F41" s="1" t="n"/>
+      <c r="G41" s="1" t="n"/>
+      <c r="H41" s="1" t="n"/>
+      <c r="I41" s="1" t="n"/>
+      <c r="J41" s="1" t="n"/>
+      <c r="K41" s="1" t="n"/>
+      <c r="L41" s="1" t="n"/>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>4. PCL mnemonic confirmed by Daniel Chin (was PLI).</t>
+          <t>1. No control group — champion/challenger placement test.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>5. Green cells are editable — change them to see recalculations.</t>
+          <t>2. Everyone gets the PCL offer — variable is WHERE they see it.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>6. MDE formula: (Za + Zb) * SQRT(p0 * (1-p0) * (1/n1 + 1/n2)).</t>
+          <t>3. Baseline RR = all-channel population-level rate (not mobile share).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>7. If reporting all 4 comparisons, consider Bonferroni correction (alpha/4 = 1.25%).</t>
+          <t>4. PCL mnemonic confirmed by Daniel Chin (was PLI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>5. Green cells are editable — change them to see recalculations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>6. MDE formula: (Za + Zb) * SQRT(p0 * (1-p0) * (1/n1 + 1/n2)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>7. With 7 comparisons, Bonferroni-adjusted alpha = 5%/7 = 0.71% per test.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B30:J30"/>
+  <mergeCells count="2">
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B32:J32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
PCL MDE: win32com recalculated, cached values prevent #VALUE! on open
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcl_mde_calculator.xlsx
+++ b/pcl_mde_calculator.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\New_projects\cards\schemas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\New_projects\cards\campaigns\PCL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC0EED7-E64D-4563-BFF4-C649C1C599A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC211F91-BB76-4C74-84DE-5EB39B42C9FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="14220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>